<commit_message>
Feat: Data Analysis and Basic Insights Return
</commit_message>
<xml_diff>
--- a/data/sales.xlsx
+++ b/data/sales.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,6 +416,9 @@
         <v>unit_price</v>
       </c>
       <c r="F1" t="str">
+        <v>cost_per_unit</v>
+      </c>
+      <c r="G1" t="str">
         <v>city</v>
       </c>
     </row>
@@ -430,12 +433,15 @@
         <v>original</v>
       </c>
       <c r="D2" t="str">
-        <v>359</v>
+        <v>35</v>
       </c>
       <c r="E2" t="str">
         <v>5.50</v>
       </c>
       <c r="F2" t="str">
+        <v>3.00</v>
+      </c>
+      <c r="G2" t="str">
         <v>Brasília</v>
       </c>
     </row>
@@ -456,6 +462,9 @@
         <v>5.50</v>
       </c>
       <c r="F3" t="str">
+        <v>2.50</v>
+      </c>
+      <c r="G3" t="str">
         <v>brasilia</v>
       </c>
     </row>
@@ -476,6 +485,9 @@
         <v>4.00</v>
       </c>
       <c r="F4" t="str">
+        <v>2.50</v>
+      </c>
+      <c r="G4" t="str">
         <v>Goiânia</v>
       </c>
     </row>
@@ -496,6 +508,9 @@
         <v>2.00</v>
       </c>
       <c r="F5" t="str">
+        <v>1.00</v>
+      </c>
+      <c r="G5" t="str">
         <v>Goiania</v>
       </c>
     </row>
@@ -513,9 +528,12 @@
         <v>49</v>
       </c>
       <c r="E6" t="str">
-        <v>6.50</v>
+        <v>7.00</v>
       </c>
       <c r="F6" t="str">
+        <v>4.00</v>
+      </c>
+      <c r="G6" t="str">
         <v>São Paulo</v>
       </c>
     </row>
@@ -527,7 +545,7 @@
         <v>soda</v>
       </c>
       <c r="C7" t="str">
-        <v>guaraná</v>
+        <v>Guaraná</v>
       </c>
       <c r="D7" t="str">
         <v>109</v>
@@ -536,7 +554,10 @@
         <v>4.50</v>
       </c>
       <c r="F7" t="str">
-        <v>sao paulo</v>
+        <v>2.40</v>
+      </c>
+      <c r="G7" t="str">
+        <v>São Paulo</v>
       </c>
     </row>
     <row r="8">
@@ -544,10 +565,10 @@
         <v>1/9/26</v>
       </c>
       <c r="B8" t="str">
-        <v>energy</v>
+        <v>energy drink</v>
       </c>
       <c r="C8" t="str">
-        <v>fusion</v>
+        <v>mosnter</v>
       </c>
       <c r="D8" t="str">
         <v>27</v>
@@ -556,12 +577,15 @@
         <v>7.50</v>
       </c>
       <c r="F8" t="str">
+        <v>3.90</v>
+      </c>
+      <c r="G8" t="str">
         <v>brasilia</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>